<commit_message>
fix: update all tailor professions to seamstress (портной -> швея)
</commit_message>
<xml_diff>
--- a/ЦНСВ БД.xlsx
+++ b/ЦНСВ БД.xlsx
@@ -630,7 +630,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -4566,7 +4566,7 @@
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" и портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E126" s="4" t="inlineStr">
@@ -4598,7 +4598,7 @@
       </c>
       <c r="D127" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" и портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E127" s="4" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="D128" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" и портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E128" s="4" t="inlineStr">
@@ -4662,7 +4662,7 @@
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" и портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E129" s="4" t="inlineStr">
@@ -7638,7 +7638,7 @@
       </c>
       <c r="D222" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="D223" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E223" s="4" t="inlineStr">
@@ -7702,7 +7702,7 @@
       </c>
       <c r="D224" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
@@ -7734,7 +7734,7 @@
       </c>
       <c r="D225" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E225" s="4" t="inlineStr">
@@ -7766,7 +7766,7 @@
       </c>
       <c r="D226" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E226" s="4" t="inlineStr">
@@ -7798,7 +7798,7 @@
       </c>
       <c r="D227" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E227" s="4" t="inlineStr">
@@ -7830,7 +7830,7 @@
       </c>
       <c r="D228" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
@@ -7862,7 +7862,7 @@
       </c>
       <c r="D229" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E229" s="4" t="inlineStr">
@@ -7894,7 +7894,7 @@
       </c>
       <c r="D230" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E230" s="4" t="inlineStr">
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D231" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E231" s="4" t="inlineStr">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="D232" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E232" s="4" t="inlineStr">
@@ -7990,7 +7990,7 @@
       </c>
       <c r="D233" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E233" s="4" t="inlineStr">
@@ -8022,7 +8022,7 @@
       </c>
       <c r="D234" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
@@ -8054,7 +8054,7 @@
       </c>
       <c r="D235" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E235" s="4" t="inlineStr">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="D236" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E236" s="4" t="inlineStr">
@@ -8118,7 +8118,7 @@
       </c>
       <c r="D237" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E237" s="4" t="inlineStr">
@@ -8150,7 +8150,7 @@
       </c>
       <c r="D238" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E238" s="4" t="inlineStr">
@@ -8182,7 +8182,7 @@
       </c>
       <c r="D239" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E239" s="4" t="inlineStr">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="D240" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E240" s="4" t="inlineStr">
@@ -8246,7 +8246,7 @@
       </c>
       <c r="D241" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E241" s="4" t="inlineStr">
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D242" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E242" s="4" t="inlineStr">
@@ -8310,7 +8310,7 @@
       </c>
       <c r="D243" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E243" s="4" t="inlineStr">
@@ -8342,7 +8342,7 @@
       </c>
       <c r="D244" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E244" s="4" t="inlineStr">
@@ -8374,7 +8374,7 @@
       </c>
       <c r="D245" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E245" s="4" t="inlineStr">
@@ -8406,7 +8406,7 @@
       </c>
       <c r="D246" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E246" s="4" t="inlineStr">
@@ -8438,7 +8438,7 @@
       </c>
       <c r="D247" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E247" s="4" t="inlineStr">
@@ -8470,7 +8470,7 @@
       </c>
       <c r="D248" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E248" s="4" t="inlineStr">
@@ -8502,7 +8502,7 @@
       </c>
       <c r="D249" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E249" s="4" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="D250" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E250" s="4" t="inlineStr">
@@ -8566,7 +8566,7 @@
       </c>
       <c r="D251" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E251" s="4" t="inlineStr">
@@ -8598,7 +8598,7 @@
       </c>
       <c r="D252" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E252" s="4" t="inlineStr">
@@ -8630,7 +8630,7 @@
       </c>
       <c r="D253" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E253" s="4" t="inlineStr">
@@ -8662,7 +8662,7 @@
       </c>
       <c r="D254" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E254" s="4" t="inlineStr">
@@ -8694,7 +8694,7 @@
       </c>
       <c r="D255" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E255" s="4" t="inlineStr">
@@ -8726,7 +8726,7 @@
       </c>
       <c r="D256" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E256" s="4" t="inlineStr">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="D257" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E257" s="4" t="inlineStr">
@@ -8790,7 +8790,7 @@
       </c>
       <c r="D258" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E258" s="4" t="inlineStr">
@@ -8822,7 +8822,7 @@
       </c>
       <c r="D259" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E259" s="4" t="inlineStr">
@@ -8854,7 +8854,7 @@
       </c>
       <c r="D260" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Портной с умением кроить" 3-4 разряда </t>
+          <t>Швея с умением кроить 3-4 разряда</t>
         </is>
       </c>
       <c r="E260" s="4" t="inlineStr">
@@ -13046,7 +13046,7 @@
       </c>
       <c r="D391" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" "Портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E391" s="4" t="inlineStr">
@@ -13078,7 +13078,7 @@
       </c>
       <c r="D392" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" "Портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E392" s="4" t="inlineStr">
@@ -13110,7 +13110,7 @@
       </c>
       <c r="D393" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" "Портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E393" s="4" t="inlineStr">
@@ -13142,7 +13142,7 @@
       </c>
       <c r="D394" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" "Портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E394" s="4" t="inlineStr">
@@ -13174,7 +13174,7 @@
       </c>
       <c r="D395" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" "Портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E395" s="4" t="inlineStr">
@@ -13206,7 +13206,7 @@
       </c>
       <c r="D396" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" "Портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E396" s="4" t="inlineStr">
@@ -13238,7 +13238,7 @@
       </c>
       <c r="D397" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" "Портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E397" s="4" t="inlineStr">
@@ -13270,7 +13270,7 @@
       </c>
       <c r="D398" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" "Портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E398" s="4" t="inlineStr">
@@ -13302,7 +13302,7 @@
       </c>
       <c r="D399" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" "Портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E399" s="4" t="inlineStr">
@@ -13334,7 +13334,7 @@
       </c>
       <c r="D400" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" "Портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E400" s="4" t="inlineStr">
@@ -13366,7 +13366,7 @@
       </c>
       <c r="D401" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" "Портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E401" s="4" t="inlineStr">
@@ -13398,7 +13398,7 @@
       </c>
       <c r="D402" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Швея" "Портной с умением кроить" </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E402" s="4" t="inlineStr">
@@ -17846,7 +17846,7 @@
       </c>
       <c r="D541" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Слесарь по ремонту автотранспортных средств" </t>
+          <t>"Слесарь по ремонту автотранспортных средств"</t>
         </is>
       </c>
       <c r="E541" s="4" t="inlineStr">
@@ -18838,7 +18838,7 @@
       </c>
       <c r="D572" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">портной,мастер народных промыслов </t>
+          <t>Швея, мастер народных промыслов</t>
         </is>
       </c>
       <c r="E572" s="4" t="inlineStr">
@@ -18870,7 +18870,7 @@
       </c>
       <c r="D573" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Слесарь по ремонту автотранспортных средств </t>
+          <t>Слесарь по ремонту автотранспортных средств</t>
         </is>
       </c>
       <c r="E573" s="4" t="inlineStr">
@@ -18902,7 +18902,7 @@
       </c>
       <c r="D574" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Слесарь по ремонту автотранспортных средств </t>
+          <t>Слесарь по ремонту автотранспортных средств</t>
         </is>
       </c>
       <c r="E574" s="4" t="inlineStr">
@@ -18934,7 +18934,7 @@
       </c>
       <c r="D575" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Слесарь по ремонту автотранспортных средств </t>
+          <t>Слесарь по ремонту автотранспортных средств</t>
         </is>
       </c>
       <c r="E575" s="4" t="inlineStr">
@@ -18966,7 +18966,7 @@
       </c>
       <c r="D576" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Слесарь по ремонту автотранспортных средств </t>
+          <t>Слесарь по ремонту автотранспортных средств</t>
         </is>
       </c>
       <c r="E576" s="4" t="inlineStr">
@@ -18998,7 +18998,7 @@
       </c>
       <c r="D577" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Слесарь по ремонту автотранспортных средств </t>
+          <t>Слесарь по ремонту автотранспортных средств</t>
         </is>
       </c>
       <c r="E577" s="4" t="inlineStr">
@@ -19346,7 +19346,7 @@
       </c>
       <c r="D588" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить </t>
+          <t>Швея с умением кроить</t>
         </is>
       </c>
       <c r="E588" s="4" t="inlineStr">
@@ -20466,7 +20466,7 @@
       </c>
       <c r="D623" s="4" t="inlineStr">
         <is>
-          <t>Портной</t>
+          <t>Швея</t>
         </is>
       </c>
       <c r="E623" s="4" t="inlineStr">
@@ -20498,7 +20498,7 @@
       </c>
       <c r="D624" s="4" t="inlineStr">
         <is>
-          <t>портной</t>
+          <t>Швея</t>
         </is>
       </c>
       <c r="E624" s="4" t="inlineStr">
@@ -20530,7 +20530,7 @@
       </c>
       <c r="D625" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">портной </t>
+          <t>Швея</t>
         </is>
       </c>
       <c r="E625" s="4" t="inlineStr">
@@ -20562,7 +20562,7 @@
       </c>
       <c r="D626" s="4" t="inlineStr">
         <is>
-          <t>портной</t>
+          <t>Швея</t>
         </is>
       </c>
       <c r="E626" s="4" t="inlineStr">
@@ -20594,7 +20594,7 @@
       </c>
       <c r="D627" s="4" t="inlineStr">
         <is>
-          <t>портной</t>
+          <t>Швея</t>
         </is>
       </c>
       <c r="E627" s="4" t="inlineStr">
@@ -20658,7 +20658,7 @@
       </c>
       <c r="D629" s="4" t="inlineStr">
         <is>
-          <t>портной</t>
+          <t>Швея</t>
         </is>
       </c>
       <c r="E629" s="4" t="inlineStr">
@@ -20690,7 +20690,7 @@
       </c>
       <c r="D630" s="4" t="inlineStr">
         <is>
-          <t>портной</t>
+          <t>Швея</t>
         </is>
       </c>
       <c r="E630" s="4" t="inlineStr">
@@ -20722,7 +20722,7 @@
       </c>
       <c r="D631" s="4" t="inlineStr">
         <is>
-          <t>портной</t>
+          <t>Швея</t>
         </is>
       </c>
       <c r="E631" s="4" t="inlineStr">
@@ -21554,7 +21554,7 @@
       </c>
       <c r="D657" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Слесерь по ремонту автотранспортных средств </t>
+          <t>Слесерь по ремонту автотранспортных средств</t>
         </is>
       </c>
       <c r="E657" s="4" t="inlineStr">
@@ -22356,7 +22356,7 @@
       </c>
       <c r="D682" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной </t>
+          <t>Швея</t>
         </is>
       </c>
       <c r="E682" s="4" t="inlineStr">
@@ -22388,7 +22388,7 @@
       </c>
       <c r="D683" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной </t>
+          <t>Швея</t>
         </is>
       </c>
       <c r="E683" s="4" t="inlineStr">
@@ -22422,7 +22422,7 @@
       </c>
       <c r="D684" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной </t>
+          <t>Швея</t>
         </is>
       </c>
       <c r="E684" s="4" t="inlineStr">
@@ -22774,7 +22774,7 @@
       </c>
       <c r="D695" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Слесарь по ремонту автотранспортных средств </t>
+          <t>Слесарь по ремонту автотранспортных средств</t>
         </is>
       </c>
       <c r="E695" s="4" t="inlineStr">
@@ -23318,7 +23318,7 @@
       </c>
       <c r="D712" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Контролер технического состояния автомототранспортных средств </t>
+          <t>Контролер технического состояния автомототранспортных средств</t>
         </is>
       </c>
       <c r="E712" s="4" t="inlineStr">
@@ -24758,7 +24758,7 @@
       </c>
       <c r="D757" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить 5 разряда </t>
+          <t>Швея с умением кроить 5 разряда</t>
         </is>
       </c>
       <c r="E757" s="4" t="inlineStr">
@@ -24790,7 +24790,7 @@
       </c>
       <c r="D758" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить 5 разряда </t>
+          <t>Швея с умением кроить 5 разряда</t>
         </is>
       </c>
       <c r="E758" s="4" t="inlineStr">
@@ -25398,7 +25398,7 @@
       </c>
       <c r="D777" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Портной с умением кроить 3 разряда </t>
+          <t>Швея с умением кроить 3 разряда</t>
         </is>
       </c>
       <c r="E777" s="4" t="inlineStr">

</xml_diff>